<commit_message>
Samarkand R10: closed themed booths (9 epochs/cities) on the plan and in the estimate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMcGkENVAoRmK9vPt9xr7W
</commit_message>
<xml_diff>
--- a/samarkand/estimate/samarkand-estimate-R10.xlsx
+++ b/samarkand/estimate/samarkand-estimate-R10.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="163">
   <si>
     <t xml:space="preserve">SAMARKAND · крытая терраса R10 — предварительная смета</t>
   </si>
@@ -261,10 +261,13 @@
     <t xml:space="preserve">Столешница из кварц-агломерата, бэк-бар без ниш</t>
   </si>
   <si>
-    <t xml:space="preserve">Кабинки: 2 скамьи, стол, резная ширма, фонарь</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ширма — фанера ЧПУ под покраску</t>
+    <t xml:space="preserve">Тематические закрытые кабинки (9 эпох): скамьи, стол, перегородки h 2,2 м, арка-портал со шторами, панно темы, потолок-шапка, свет, вентилятор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">средняя; мурал и резьба дороже, текстиль дешевле</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Панно — печать на ткани, резьба ЧПУ из МДФ</t>
   </si>
   <si>
     <t xml:space="preserve">Айван: седир-кабинки на 6 (2 скамьи 1,85 м, стол 1600×700, резная перегородка h 1200, фонарь)</t>
@@ -2337,7 +2340,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="n">
         <v>29</v>
       </c>
@@ -2351,26 +2354,28 @@
         <v>9</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>16000000</v>
+        <v>30000000</v>
       </c>
       <c r="F46" s="13" t="n">
         <f aca="false">D46*E46</f>
-        <v>144000000</v>
+        <v>270000000</v>
       </c>
       <c r="G46" s="13" t="n">
         <f aca="false">F46/$H$2</f>
-        <v>5538.46153846154</v>
-      </c>
-      <c r="H46" s="11"/>
+        <v>10384.6153846154</v>
+      </c>
+      <c r="H46" s="11" t="s">
+        <v>80</v>
+      </c>
       <c r="I46" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J46" s="13" t="n">
-        <v>12500000</v>
+        <v>22000000</v>
       </c>
       <c r="K46" s="13" t="n">
         <f aca="false">D46*J46</f>
-        <v>112500000</v>
+        <v>198000000</v>
       </c>
       <c r="L46" s="8"/>
     </row>
@@ -2379,7 +2384,7 @@
         <v>30</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C47" s="10" t="s">
         <v>36</v>
@@ -2400,7 +2405,7 @@
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J47" s="13" t="n">
         <v>17000000</v>
@@ -2416,7 +2421,7 @@
         <v>31</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C48" s="10" t="s">
         <v>36</v>
@@ -2449,7 +2454,7 @@
         <v>32</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C49" s="10" t="s">
         <v>36</v>
@@ -2470,7 +2475,7 @@
       </c>
       <c r="H49" s="11"/>
       <c r="I49" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J49" s="13" t="n">
         <v>45000000</v>
@@ -2486,7 +2491,7 @@
         <v>33</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C50" s="10" t="s">
         <v>17</v>
@@ -2519,7 +2524,7 @@
         <v>34</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C51" s="10" t="s">
         <v>36</v>
@@ -2552,7 +2557,7 @@
         <v>35</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C52" s="10" t="s">
         <v>17</v>
@@ -2573,7 +2578,7 @@
       </c>
       <c r="H52" s="11"/>
       <c r="I52" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J52" s="13" t="n">
         <v>35000000</v>
@@ -2589,7 +2594,7 @@
         <v>36</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" s="10" t="s">
         <v>17</v>
@@ -2622,7 +2627,7 @@
         <v>37</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C54" s="10" t="s">
         <v>17</v>
@@ -2655,7 +2660,7 @@
         <v>38</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C55" s="10" t="s">
         <v>17</v>
@@ -2676,7 +2681,7 @@
       </c>
       <c r="H55" s="11"/>
       <c r="I55" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J55" s="13" t="n">
         <v>42000000</v>
@@ -2692,7 +2697,7 @@
         <v>39</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>17</v>
@@ -2712,7 +2717,7 @@
         <v>2000</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I56" s="11"/>
       <c r="J56" s="13"/>
@@ -2727,7 +2732,7 @@
         <v>40</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C57" s="10" t="s">
         <v>17</v>
@@ -2760,7 +2765,7 @@
         <v>41</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C58" s="10" t="s">
         <v>17</v>
@@ -2791,25 +2796,25 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
       <c r="B59" s="15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C59" s="14"/>
       <c r="D59" s="16"/>
       <c r="E59" s="17"/>
       <c r="F59" s="18" t="n">
         <f aca="false">SUM(F45:F58)</f>
-        <v>1006000000</v>
+        <v>1132000000</v>
       </c>
       <c r="G59" s="18" t="n">
         <f aca="false">F59/$H$2</f>
-        <v>38692.3076923077</v>
+        <v>43538.4615384615</v>
       </c>
       <c r="H59" s="19"/>
       <c r="I59" s="19"/>
       <c r="J59" s="17"/>
       <c r="K59" s="18" t="n">
         <f aca="false">SUM(K45:K58)</f>
-        <v>848500000</v>
+        <v>934000000</v>
       </c>
       <c r="L59" s="8"/>
     </row>
@@ -2827,7 +2832,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="8"/>
@@ -2844,7 +2849,7 @@
         <v>42</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C62" s="10" t="s">
         <v>36</v>
@@ -2864,10 +2869,10 @@
         <v>3123.07692307692</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J62" s="13" t="n">
         <v>2100000</v>
@@ -2883,7 +2888,7 @@
         <v>43</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C63" s="10" t="s">
         <v>36</v>
@@ -2904,7 +2909,7 @@
       </c>
       <c r="H63" s="11"/>
       <c r="I63" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J63" s="13" t="n">
         <v>1150000</v>
@@ -2920,7 +2925,7 @@
         <v>44</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C64" s="10" t="s">
         <v>36</v>
@@ -2951,7 +2956,7 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
       <c r="B65" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C65" s="14"/>
       <c r="D65" s="16"/>
@@ -2987,7 +2992,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="8"/>
@@ -3004,7 +3009,7 @@
         <v>45</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C68" s="10" t="s">
         <v>21</v>
@@ -3037,7 +3042,7 @@
         <v>46</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C69" s="10" t="s">
         <v>17</v>
@@ -3057,10 +3062,10 @@
         <v>6346.15384615385</v>
       </c>
       <c r="H69" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J69" s="13" t="n">
         <v>120000000</v>
@@ -3076,7 +3081,7 @@
         <v>47</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C70" s="10" t="s">
         <v>36</v>
@@ -3096,7 +3101,7 @@
         <v>2215.38461538462</v>
       </c>
       <c r="H70" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I70" s="11"/>
       <c r="J70" s="13"/>
@@ -3111,7 +3116,7 @@
         <v>48</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C71" s="10" t="s">
         <v>17</v>
@@ -3144,7 +3149,7 @@
         <v>49</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C72" s="10" t="s">
         <v>17</v>
@@ -3175,7 +3180,7 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
       <c r="B73" s="15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C73" s="14"/>
       <c r="D73" s="16"/>
@@ -3211,7 +3216,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D75" s="7"/>
       <c r="E75" s="8"/>
@@ -3225,7 +3230,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>17</v>
@@ -3257,7 +3262,7 @@
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
       <c r="B77" s="15" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C77" s="14"/>
       <c r="D77" s="16"/>
@@ -3293,53 +3298,53 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D79" s="7"/>
       <c r="E79" s="8"/>
       <c r="F79" s="8" t="n">
         <f aca="false">F9+F19+F28+F42+F59+F65+F73+F77</f>
-        <v>3534949000</v>
+        <v>3660949000</v>
       </c>
       <c r="G79" s="8" t="n">
         <f aca="false">F79/$H$2</f>
-        <v>135959.576923077</v>
+        <v>140805.730769231</v>
       </c>
       <c r="H79" s="9"/>
       <c r="I79" s="9"/>
       <c r="J79" s="8"/>
       <c r="K79" s="8" t="n">
         <f aca="false">K9+K19+K28+K42+K59+K65+K73+K77</f>
-        <v>3053711000</v>
+        <v>3139211000</v>
       </c>
       <c r="L79" s="8"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D80" s="7"/>
       <c r="E80" s="8"/>
       <c r="F80" s="8" t="n">
         <f aca="false">F79*0.1</f>
-        <v>353494900</v>
+        <v>366094900</v>
       </c>
       <c r="G80" s="8" t="n">
         <f aca="false">F80/$H$2</f>
-        <v>13595.9576923077</v>
+        <v>14080.5730769231</v>
       </c>
       <c r="H80" s="9"/>
       <c r="I80" s="9"/>
       <c r="J80" s="8"/>
       <c r="K80" s="8" t="n">
         <f aca="false">K79*0.1</f>
-        <v>305371100</v>
+        <v>313921100</v>
       </c>
       <c r="L80" s="8"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D81" s="7"/>
       <c r="E81" s="8"/>
@@ -3362,29 +3367,29 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="21"/>
       <c r="B82" s="22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C82" s="21"/>
       <c r="D82" s="23"/>
       <c r="E82" s="24"/>
       <c r="F82" s="24" t="n">
         <f aca="false">SUM(F79:F81)</f>
-        <v>3933443900</v>
+        <v>4072043900</v>
       </c>
       <c r="G82" s="24" t="n">
         <f aca="false">F82/$H$2</f>
-        <v>151286.303846154</v>
+        <v>156617.073076923</v>
       </c>
       <c r="H82" s="22"/>
       <c r="I82" s="22"/>
       <c r="J82" s="24"/>
       <c r="K82" s="24" t="n">
         <f aca="false">SUM(K79:K81)</f>
-        <v>3404082100</v>
+        <v>3498132100</v>
       </c>
       <c r="L82" s="24" t="n">
         <f aca="false">K82/$H$2</f>
-        <v>130926.234615385</v>
+        <v>134543.542307692</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,13 +3406,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D84" s="7"/>
       <c r="E84" s="8"/>
       <c r="F84" s="25" t="n">
         <f aca="false">F82-K82</f>
-        <v>529361800</v>
+        <v>573911800</v>
       </c>
       <c r="G84" s="8"/>
       <c r="H84" s="9"/>
@@ -3418,13 +3423,13 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D85" s="7"/>
       <c r="E85" s="8"/>
       <c r="F85" s="8" t="n">
         <f aca="false">F82/446.5</f>
-        <v>8809504.81522956</v>
+        <v>9119919.14893617</v>
       </c>
       <c r="G85" s="8"/>
       <c r="H85" s="9"/>
@@ -3435,13 +3440,13 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="8"/>
       <c r="F86" s="8" t="n">
         <f aca="false">F82/175</f>
-        <v>22476822.2857143</v>
+        <v>23268822.2857143</v>
       </c>
       <c r="G86" s="8"/>
       <c r="H86" s="9"/>
@@ -3452,22 +3457,22 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -3499,12 +3504,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>5</v>
@@ -3524,7 +3529,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>36</v>
@@ -3540,12 +3545,12 @@
         <v>28000000</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>36</v>
@@ -3563,7 +3568,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B6" s="0" t="s">
         <v>17</v>
@@ -3581,7 +3586,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>17</v>
@@ -3597,12 +3602,12 @@
         <v>88000000</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>36</v>
@@ -3620,7 +3625,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>17</v>
@@ -3638,7 +3643,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>17</v>
@@ -3656,7 +3661,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>17</v>
@@ -3674,7 +3679,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B12" s="0" t="s">
         <v>17</v>
@@ -3692,7 +3697,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>17</v>
@@ -3710,7 +3715,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>17</v>
@@ -3728,7 +3733,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>17</v>
@@ -3746,7 +3751,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>17</v>
@@ -3764,7 +3769,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>17</v>
@@ -3782,7 +3787,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E18" s="29" t="n">
         <f aca="false">SUM(E4:E17)</f>
@@ -3813,7 +3818,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="0" t="n">
         <v>446.5</v>
@@ -3824,7 +3829,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>419.5</v>
@@ -3835,7 +3840,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>27</v>
@@ -3846,7 +3851,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>9.8</v>
@@ -3857,7 +3862,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>285.7</v>
@@ -3868,7 +3873,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>49.3</v>
@@ -3879,7 +3884,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>15.8</v>
@@ -3890,7 +3895,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>20.2</v>
@@ -3901,7 +3906,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>28</v>
@@ -3912,7 +3917,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>56</v>
@@ -3923,7 +3928,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>175</v>
@@ -3931,7 +3936,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>21.2</v>

</xml_diff>